<commit_message>
fixed second merging of labels for cell data
</commit_message>
<xml_diff>
--- a/annotation/Species_list_vs_CATAMI_2023_01.xlsx
+++ b/annotation/Species_list_vs_CATAMI_2023_01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jjansen\Desktop\science\SouthernOceanBiodiversityMapping\ARC_Data\annotation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99CD8A5B-5DD6-4A12-A0D2-B75294CF0B48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1559BFAB-B48F-464E-AEC0-F3DBFADD243F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15030" yWindow="-18120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1002" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1009" uniqueCount="479">
   <si>
     <t>Label</t>
   </si>
@@ -1455,6 +1455,9 @@
   </si>
   <si>
     <t>Sponge_Erect_Other</t>
+  </si>
+  <si>
+    <t>Molluscs_Gastropods</t>
   </si>
 </sst>
 </file>
@@ -4232,6 +4235,9 @@
       <c r="J59" s="5" t="s">
         <v>473</v>
       </c>
+      <c r="K59" t="s">
+        <v>70</v>
+      </c>
       <c r="L59">
         <v>5</v>
       </c>
@@ -4240,6 +4246,9 @@
       </c>
       <c r="N59" s="5" t="s">
         <v>473</v>
+      </c>
+      <c r="O59" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.3">
@@ -4507,6 +4516,9 @@
       <c r="N65" s="5" t="s">
         <v>473</v>
       </c>
+      <c r="O65" t="s">
+        <v>478</v>
+      </c>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
@@ -4551,6 +4563,9 @@
       <c r="N66" s="5" t="s">
         <v>473</v>
       </c>
+      <c r="O66" t="s">
+        <v>478</v>
+      </c>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
@@ -4595,6 +4610,9 @@
       <c r="N67" s="5" t="s">
         <v>473</v>
       </c>
+      <c r="O67" t="s">
+        <v>478</v>
+      </c>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
@@ -5176,6 +5194,9 @@
       <c r="M83">
         <v>2.5999999999999999E-2</v>
       </c>
+      <c r="O83" t="s">
+        <v>476</v>
+      </c>
     </row>
     <row r="84" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
@@ -5213,6 +5234,9 @@
       </c>
       <c r="M84">
         <v>0.02</v>
+      </c>
+      <c r="O84" t="s">
+        <v>476</v>
       </c>
     </row>
     <row r="85" spans="1:15" x14ac:dyDescent="0.3">

</xml_diff>